<commit_message>
test: the DataValidation example's copied list now refers to the copy (#525)
Examples/Misc/DataValidation copies a sheet whose A5 is List(ws.Range("C1:C2")). The copy used to save it in x14 as 'Data Validation'!$C$1:$C$2, the original sheet; it now saves $C$1:$C$2 in the standard form, the copy's own cells, as Excel's copy does in dv-copy-after.xlsx. sheet3.xml is the only part that differs.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Misc/DataValidation.xlsx
+++ b/XLibur.Tests/Resource/Examples/Misc/DataValidation.xlsx
@@ -679,7 +679,7 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="6">
+  <x:dataValidations count="7">
     <x:dataValidation type="decimal" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A1:A1">
       <x:formula1>1</x:formula1>
       <x:formula2>5</x:formula2>
@@ -690,6 +690,10 @@
     </x:dataValidation>
     <x:dataValidation type="date" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="Can't party like it's 1999." prompt="Please enter a date in this century." sqref="A4:A4">
       <x:formula1>36526</x:formula1>
+      <x:formula2/>
+    </x:dataValidation>
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A5:A5">
+      <x:formula1>$C$1:$C$2</x:formula1>
       <x:formula2/>
     </x:dataValidation>
     <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
@@ -717,18 +721,6 @@
     <x:firstFooter/>
   </x:headerFooter>
   <x:tableParts count="0"/>
-  <x:extLst>
-    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="">
-          <x14:formula1>
-            <xm:f>'Data Validation'!$C$1:$C$2</xm:f>
-          </x14:formula1>
-          <xm:sqref>A5:A5</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </x:ext>
-  </x:extLst>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: a data validation criterion set with a leading equals sign is saved without it (#523)
DataValidationWriter.UsesExternalSheet chose between the standard element and the x14 extension with XLHelper.IsValidRangeAddress, which allows no leading equals sign, so a list set as an equals sign followed by Data!A1:A3 was written with the sign inside formula1, and in the standard form. The writer now takes the sign off with FormulaText.WithoutLeadingEquals before it decides, so the rule is written as Excel writes it: in x14:dataValidation for a range on another sheet, and without the sheet name for a range on its own sheet. MinValue, MaxValue and Value still return the text as it was set. Tests that pinned the sign in the saved file now expect the text Excel writes, and the DataValidation example reference file loses the sign before YesNo and nothing else.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Misc/DataValidation.xlsx
+++ b/XLibur.Tests/Resource/Examples/Misc/DataValidation.xlsx
@@ -505,7 +505,7 @@
       <x:formula2/>
     </x:dataValidation>
     <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
-      <x:formula1>=YesNo</x:formula1>
+      <x:formula1>YesNo</x:formula1>
       <x:formula2/>
     </x:dataValidation>
     <x:dataValidation type="whole" errorStyle="stop" operator="equal" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="B1:B2">
@@ -697,7 +697,7 @@
       <x:formula2/>
     </x:dataValidation>
     <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
-      <x:formula1>=YesNo</x:formula1>
+      <x:formula1>YesNo</x:formula1>
       <x:formula2/>
     </x:dataValidation>
     <x:dataValidation type="whole" errorStyle="stop" operator="equal" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="B1:B2">
@@ -899,7 +899,7 @@
       <x:formula2/>
     </x:dataValidation>
     <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
-      <x:formula1>=YesNo</x:formula1>
+      <x:formula1>YesNo</x:formula1>
       <x:formula2/>
     </x:dataValidation>
     <x:dataValidation type="whole" errorStyle="stop" operator="equal" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="B1:B2">

</xml_diff>